<commit_message>
Feat: Problem 2 rearrange 0 and 1
</commit_message>
<xml_diff>
--- a/DSA Pattern sheets.xlsx
+++ b/DSA Pattern sheets.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="361">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="362">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -48,6 +48,9 @@
   </si>
   <si>
     <t>1. Pattern: Two Pointers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Solved </t>
   </si>
   <si>
     <t>Pair with Target Sum (easy)</t>
@@ -2648,30 +2651,32 @@
       <c r="E3" s="7"/>
       <c r="F3" s="7"/>
     </row>
-    <row r="4" ht="15.15" spans="1:6">
+    <row r="4" spans="1:6">
       <c r="A4" s="4">
         <v>4</v>
       </c>
-      <c r="B4" s="5"/>
+      <c r="B4" s="5" t="s">
+        <v>7</v>
+      </c>
       <c r="C4" s="8" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E4" s="7"/>
       <c r="F4" s="7"/>
     </row>
-    <row r="5" ht="15.15" spans="1:6">
+    <row r="5" spans="1:6">
       <c r="A5" s="4">
         <v>5</v>
       </c>
       <c r="B5" s="5"/>
       <c r="C5" s="8" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E5" s="8"/>
       <c r="F5" s="5"/>
@@ -2682,16 +2687,16 @@
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" ht="15.15" spans="1:6">
@@ -2700,10 +2705,10 @@
       </c>
       <c r="B7" s="5"/>
       <c r="C7" s="8" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E7" s="7"/>
       <c r="F7" s="7"/>
@@ -2714,10 +2719,10 @@
       </c>
       <c r="B8" s="5"/>
       <c r="C8" s="8" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E8" s="7"/>
       <c r="F8" s="7"/>
@@ -2728,10 +2733,10 @@
       </c>
       <c r="B9" s="5"/>
       <c r="C9" s="8" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E9" s="7"/>
       <c r="F9" s="7"/>
@@ -2742,10 +2747,10 @@
       </c>
       <c r="B10" s="5"/>
       <c r="C10" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E10" s="7"/>
       <c r="F10" s="7"/>
@@ -2756,10 +2761,10 @@
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E11" s="7"/>
       <c r="F11" s="7"/>
@@ -2770,10 +2775,10 @@
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="8" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E12" s="7"/>
       <c r="F12" s="7"/>
@@ -2784,10 +2789,10 @@
       </c>
       <c r="B13" s="5"/>
       <c r="C13" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E13" s="7"/>
       <c r="F13" s="7"/>
@@ -2798,10 +2803,10 @@
       </c>
       <c r="B14" s="5"/>
       <c r="C14" s="5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E14" s="7"/>
       <c r="F14" s="7"/>
@@ -2812,13 +2817,13 @@
       </c>
       <c r="B15" s="5"/>
       <c r="C15" s="5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F15" s="10"/>
     </row>
@@ -2828,7 +2833,7 @@
       </c>
       <c r="B16" s="5"/>
       <c r="C16" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D16" s="7"/>
       <c r="E16" s="7"/>
@@ -2840,10 +2845,10 @@
       </c>
       <c r="B17" s="5"/>
       <c r="C17" s="8" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E17" s="7"/>
       <c r="F17" s="7"/>
@@ -2854,10 +2859,10 @@
       </c>
       <c r="B18" s="5"/>
       <c r="C18" s="8" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E18" s="7"/>
       <c r="F18" s="7"/>
@@ -2868,10 +2873,10 @@
       </c>
       <c r="B19" s="5"/>
       <c r="C19" s="8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E19" s="7"/>
       <c r="F19" s="7"/>
@@ -2882,10 +2887,10 @@
       </c>
       <c r="B20" s="5"/>
       <c r="C20" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D20" s="10" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E20" s="7"/>
       <c r="F20" s="7"/>
@@ -2896,10 +2901,10 @@
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="8" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E21" s="7"/>
       <c r="F21" s="7"/>
@@ -2910,10 +2915,10 @@
       </c>
       <c r="B22" s="5"/>
       <c r="C22" s="5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D22" s="10" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E22" s="7"/>
       <c r="F22" s="7"/>
@@ -2924,10 +2929,10 @@
       </c>
       <c r="B23" s="5"/>
       <c r="C23" s="5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E23" s="7"/>
       <c r="F23" s="7"/>
@@ -2938,10 +2943,10 @@
       </c>
       <c r="B24" s="5"/>
       <c r="C24" s="5" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D24" s="10" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E24" s="7"/>
       <c r="F24" s="7"/>
@@ -2952,7 +2957,7 @@
       </c>
       <c r="B25" s="5"/>
       <c r="C25" s="6" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D25" s="7"/>
       <c r="E25" s="7"/>
@@ -2964,10 +2969,10 @@
       </c>
       <c r="B26" s="5"/>
       <c r="C26" s="8" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E26" s="7"/>
       <c r="F26" s="7"/>
@@ -2978,10 +2983,10 @@
       </c>
       <c r="B27" s="5"/>
       <c r="C27" s="8" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E27" s="7"/>
       <c r="F27" s="7"/>
@@ -2992,10 +2997,10 @@
       </c>
       <c r="B28" s="5"/>
       <c r="C28" s="8" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D28" s="10" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E28" s="7"/>
       <c r="F28" s="7"/>
@@ -3006,10 +3011,10 @@
       </c>
       <c r="B29" s="5"/>
       <c r="C29" s="8" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D29" s="10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E29" s="7"/>
       <c r="F29" s="7"/>
@@ -3020,10 +3025,10 @@
       </c>
       <c r="B30" s="5"/>
       <c r="C30" s="8" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D30" s="10" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E30" s="7"/>
       <c r="F30" s="7"/>
@@ -3034,10 +3039,10 @@
       </c>
       <c r="B31" s="5"/>
       <c r="C31" s="8" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D31" s="10" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E31" s="7"/>
       <c r="F31" s="7"/>
@@ -3048,10 +3053,10 @@
       </c>
       <c r="B32" s="5"/>
       <c r="C32" s="8" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D32" s="10" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E32" s="7"/>
       <c r="F32" s="7"/>
@@ -3062,10 +3067,10 @@
       </c>
       <c r="B33" s="5"/>
       <c r="C33" s="8" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D33" s="10" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E33" s="7"/>
       <c r="F33" s="7"/>
@@ -3076,10 +3081,10 @@
       </c>
       <c r="B34" s="5"/>
       <c r="C34" s="8" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D34" s="11" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E34" s="7"/>
       <c r="F34" s="7"/>
@@ -3090,10 +3095,10 @@
       </c>
       <c r="B35" s="5"/>
       <c r="C35" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D35" s="10" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E35" s="7"/>
       <c r="F35" s="7"/>
@@ -3104,10 +3109,10 @@
       </c>
       <c r="B36" s="5"/>
       <c r="C36" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D36" s="10" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E36" s="7"/>
       <c r="F36" s="7"/>
@@ -3118,10 +3123,10 @@
       </c>
       <c r="B37" s="5"/>
       <c r="C37" s="5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D37" s="10" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E37" s="7"/>
       <c r="F37" s="7"/>
@@ -3132,7 +3137,7 @@
       </c>
       <c r="B38" s="5"/>
       <c r="C38" s="6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D38" s="7"/>
       <c r="E38" s="7"/>
@@ -3144,10 +3149,10 @@
       </c>
       <c r="B39" s="5"/>
       <c r="C39" s="12" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D39" s="7" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E39" s="7"/>
       <c r="F39" s="7"/>
@@ -3158,10 +3163,10 @@
       </c>
       <c r="B40" s="5"/>
       <c r="C40" s="8" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D40" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E40" s="7"/>
       <c r="F40" s="7"/>
@@ -3172,10 +3177,10 @@
       </c>
       <c r="B41" s="5"/>
       <c r="C41" s="12" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D41" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E41" s="7"/>
       <c r="F41" s="7"/>
@@ -3186,10 +3191,10 @@
       </c>
       <c r="B42" s="5"/>
       <c r="C42" s="12" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D42" s="7" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E42" s="7"/>
       <c r="F42" s="7"/>
@@ -3200,10 +3205,10 @@
       </c>
       <c r="B43" s="5"/>
       <c r="C43" s="12" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D43" s="7" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E43" s="7"/>
       <c r="F43" s="7"/>
@@ -3214,10 +3219,10 @@
       </c>
       <c r="B44" s="5"/>
       <c r="C44" s="12" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D44" s="13" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E44" s="7"/>
       <c r="F44" s="7"/>
@@ -3228,7 +3233,7 @@
       </c>
       <c r="B45" s="5"/>
       <c r="C45" s="6" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D45" s="7"/>
       <c r="E45" s="7"/>
@@ -3240,10 +3245,10 @@
       </c>
       <c r="B46" s="5"/>
       <c r="C46" s="12" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D46" s="7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E46" s="7"/>
       <c r="F46" s="7"/>
@@ -3254,10 +3259,10 @@
       </c>
       <c r="B47" s="5"/>
       <c r="C47" s="12" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D47" s="7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E47" s="7"/>
       <c r="F47" s="7"/>
@@ -3268,10 +3273,10 @@
       </c>
       <c r="B48" s="5"/>
       <c r="C48" s="12" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D48" s="7" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E48" s="7"/>
       <c r="F48" s="7"/>
@@ -3282,10 +3287,10 @@
       </c>
       <c r="B49" s="5"/>
       <c r="C49" s="12" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D49" s="7" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E49" s="7"/>
       <c r="F49" s="7"/>
@@ -3296,10 +3301,10 @@
       </c>
       <c r="B50" s="5"/>
       <c r="C50" s="14" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D50" s="7" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E50" s="7"/>
       <c r="F50" s="7"/>
@@ -3310,10 +3315,10 @@
       </c>
       <c r="B51" s="5"/>
       <c r="C51" s="14" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D51" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E51" s="7"/>
       <c r="F51" s="7"/>
@@ -3324,7 +3329,7 @@
       </c>
       <c r="B52" s="5"/>
       <c r="C52" s="6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D52" s="7"/>
       <c r="E52" s="7"/>
@@ -3336,10 +3341,10 @@
       </c>
       <c r="B53" s="5"/>
       <c r="C53" s="8" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D53" s="10" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E53" s="7"/>
       <c r="F53" s="7"/>
@@ -3350,10 +3355,10 @@
       </c>
       <c r="B54" s="5"/>
       <c r="C54" s="8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D54" s="10" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E54" s="7"/>
       <c r="F54" s="7"/>
@@ -3364,10 +3369,10 @@
       </c>
       <c r="B55" s="5"/>
       <c r="C55" s="8" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D55" s="10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E55" s="7"/>
       <c r="F55" s="7"/>
@@ -3378,10 +3383,10 @@
       </c>
       <c r="B56" s="5"/>
       <c r="C56" s="8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D56" s="10" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E56" s="10"/>
       <c r="F56" s="7"/>
@@ -3392,10 +3397,10 @@
       </c>
       <c r="B57" s="5"/>
       <c r="C57" s="8" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D57" s="10" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E57" s="7"/>
       <c r="F57" s="7"/>
@@ -3406,10 +3411,10 @@
       </c>
       <c r="B58" s="5"/>
       <c r="C58" s="5" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D58" s="10" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E58" s="7"/>
       <c r="F58" s="7"/>
@@ -3420,10 +3425,10 @@
       </c>
       <c r="B59" s="5"/>
       <c r="C59" s="5" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D59" s="10" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E59" s="7"/>
       <c r="F59" s="7"/>
@@ -3434,7 +3439,7 @@
       </c>
       <c r="B60" s="5"/>
       <c r="C60" s="6" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D60" s="7"/>
       <c r="E60" s="7"/>
@@ -3446,10 +3451,10 @@
       </c>
       <c r="B61" s="5"/>
       <c r="C61" s="8" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D61" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E61" s="7"/>
       <c r="F61" s="7"/>
@@ -3460,10 +3465,10 @@
       </c>
       <c r="B62" s="5"/>
       <c r="C62" s="8" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D62" s="10" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E62" s="7"/>
       <c r="F62" s="7"/>
@@ -3474,10 +3479,10 @@
       </c>
       <c r="B63" s="5"/>
       <c r="C63" s="8" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D63" s="10" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E63" s="7"/>
       <c r="F63" s="7"/>
@@ -3488,10 +3493,10 @@
       </c>
       <c r="B64" s="5"/>
       <c r="C64" s="8" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D64" s="10" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E64" s="7"/>
       <c r="F64" s="7"/>
@@ -3502,10 +3507,10 @@
       </c>
       <c r="B65" s="5"/>
       <c r="C65" s="5" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D65" s="10" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E65" s="7"/>
       <c r="F65" s="7"/>
@@ -3516,10 +3521,10 @@
       </c>
       <c r="B66" s="5"/>
       <c r="C66" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D66" s="10" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E66" s="7"/>
       <c r="F66" s="7"/>
@@ -3530,7 +3535,7 @@
       </c>
       <c r="B67" s="5"/>
       <c r="C67" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D67" s="7"/>
       <c r="E67" s="7"/>
@@ -3542,10 +3547,10 @@
       </c>
       <c r="B68" s="5"/>
       <c r="C68" s="8" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D68" s="10" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E68" s="7"/>
       <c r="F68" s="7"/>
@@ -3556,10 +3561,10 @@
       </c>
       <c r="B69" s="5"/>
       <c r="C69" s="8" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D69" s="10" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E69" s="7"/>
       <c r="F69" s="7"/>
@@ -3570,7 +3575,7 @@
       </c>
       <c r="B70" s="5"/>
       <c r="C70" s="8" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D70" s="7"/>
       <c r="E70" s="7"/>
@@ -3582,10 +3587,10 @@
       </c>
       <c r="B71" s="5"/>
       <c r="C71" s="8" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D71" s="10" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E71" s="5"/>
       <c r="F71" s="5"/>
@@ -3596,10 +3601,10 @@
       </c>
       <c r="B72" s="5"/>
       <c r="C72" s="8" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D72" s="10" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E72" s="7"/>
       <c r="F72" s="7"/>
@@ -3610,10 +3615,10 @@
       </c>
       <c r="B73" s="5"/>
       <c r="C73" s="5" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D73" s="10" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E73" s="7"/>
       <c r="F73" s="7"/>
@@ -3624,10 +3629,10 @@
       </c>
       <c r="B74" s="5"/>
       <c r="C74" s="8" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D74" s="10" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E74" s="7"/>
       <c r="F74" s="7"/>
@@ -3638,10 +3643,10 @@
       </c>
       <c r="B75" s="5"/>
       <c r="C75" s="5" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D75" s="10" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E75" s="7"/>
       <c r="F75" s="7"/>
@@ -3652,10 +3657,10 @@
       </c>
       <c r="B76" s="5"/>
       <c r="C76" s="5" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D76" s="10" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E76" s="7"/>
       <c r="F76" s="7"/>
@@ -3666,7 +3671,7 @@
       </c>
       <c r="B77" s="5"/>
       <c r="C77" s="6" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D77" s="7"/>
       <c r="E77" s="7"/>
@@ -3678,10 +3683,10 @@
       </c>
       <c r="B78" s="5"/>
       <c r="C78" s="8" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D78" s="10" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E78" s="7"/>
       <c r="F78" s="7"/>
@@ -3692,10 +3697,10 @@
       </c>
       <c r="B79" s="5"/>
       <c r="C79" s="8" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D79" s="10" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E79" s="7"/>
       <c r="F79" s="7"/>
@@ -3706,10 +3711,10 @@
       </c>
       <c r="B80" s="5"/>
       <c r="C80" s="8" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D80" s="10" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E80" s="7"/>
       <c r="F80" s="7"/>
@@ -3720,10 +3725,10 @@
       </c>
       <c r="B81" s="5"/>
       <c r="C81" s="8" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D81" s="10" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E81" s="7"/>
       <c r="F81" s="7"/>
@@ -3734,7 +3739,7 @@
       </c>
       <c r="B82" s="5"/>
       <c r="C82" s="6" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D82" s="15"/>
       <c r="E82" s="7"/>
@@ -3746,10 +3751,10 @@
       </c>
       <c r="B83" s="5"/>
       <c r="C83" s="8" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D83" s="10" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E83" s="7"/>
       <c r="F83" s="7"/>
@@ -3760,10 +3765,10 @@
       </c>
       <c r="B84" s="5"/>
       <c r="C84" s="8" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D84" s="10" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E84" s="7"/>
       <c r="F84" s="7"/>
@@ -3774,10 +3779,10 @@
       </c>
       <c r="B85" s="5"/>
       <c r="C85" s="8" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D85" s="10" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E85" s="7"/>
       <c r="F85" s="7"/>
@@ -3788,10 +3793,10 @@
       </c>
       <c r="B86" s="5"/>
       <c r="C86" s="8" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D86" s="10" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E86" s="7"/>
       <c r="F86" s="7"/>
@@ -3802,10 +3807,10 @@
       </c>
       <c r="B87" s="5"/>
       <c r="C87" s="5" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D87" s="10" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E87" s="7"/>
       <c r="F87" s="7"/>
@@ -3816,10 +3821,10 @@
       </c>
       <c r="B88" s="5"/>
       <c r="C88" s="8" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D88" s="10" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E88" s="7"/>
       <c r="F88" s="7"/>
@@ -3830,10 +3835,10 @@
       </c>
       <c r="B89" s="5"/>
       <c r="C89" s="5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D89" s="10" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="E89" s="7"/>
       <c r="F89" s="7"/>
@@ -3844,10 +3849,10 @@
       </c>
       <c r="B90" s="5"/>
       <c r="C90" s="8" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D90" s="10" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="E90" s="7"/>
       <c r="F90" s="7"/>
@@ -3858,10 +3863,10 @@
       </c>
       <c r="B91" s="5"/>
       <c r="C91" s="8" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D91" s="10" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E91" s="7"/>
       <c r="F91" s="7"/>
@@ -3872,10 +3877,10 @@
       </c>
       <c r="B92" s="5"/>
       <c r="C92" s="8" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D92" s="10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="E92" s="7"/>
       <c r="F92" s="7"/>
@@ -3886,10 +3891,10 @@
       </c>
       <c r="B93" s="5"/>
       <c r="C93" s="8" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D93" s="10" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="E93" s="7"/>
       <c r="F93" s="7"/>
@@ -3900,10 +3905,10 @@
       </c>
       <c r="B94" s="5"/>
       <c r="C94" s="5" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D94" s="10" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="E94" s="7"/>
       <c r="F94" s="7"/>
@@ -3914,10 +3919,10 @@
       </c>
       <c r="B95" s="5"/>
       <c r="C95" s="8" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D95" s="10" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="E95" s="7"/>
       <c r="F95" s="7"/>
@@ -3928,10 +3933,10 @@
       </c>
       <c r="B96" s="5"/>
       <c r="C96" s="5" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D96" s="10" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="E96" s="7"/>
       <c r="F96" s="7"/>
@@ -3942,10 +3947,10 @@
       </c>
       <c r="B97" s="5"/>
       <c r="C97" s="5" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D97" s="10" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="E97" s="7"/>
       <c r="F97" s="7"/>
@@ -3956,10 +3961,10 @@
       </c>
       <c r="B98" s="5"/>
       <c r="C98" s="5" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="D98" s="10" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="E98" s="7"/>
       <c r="F98" s="7"/>
@@ -3970,10 +3975,10 @@
       </c>
       <c r="B99" s="5"/>
       <c r="C99" s="8" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D99" s="10" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="E99" s="7"/>
       <c r="F99" s="7"/>
@@ -3984,10 +3989,10 @@
       </c>
       <c r="B100" s="5"/>
       <c r="C100" s="5" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D100" s="10" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="E100" s="7"/>
       <c r="F100" s="7"/>
@@ -3998,10 +4003,10 @@
       </c>
       <c r="B101" s="5"/>
       <c r="C101" s="8" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="D101" s="10" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E101" s="7"/>
       <c r="F101" s="7"/>
@@ -4012,10 +4017,10 @@
       </c>
       <c r="B102" s="5"/>
       <c r="C102" s="8" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D102" s="10" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="E102" s="7"/>
       <c r="F102" s="7"/>
@@ -4026,10 +4031,10 @@
       </c>
       <c r="B103" s="5"/>
       <c r="C103" s="8" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D103" s="10" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="E103" s="7"/>
       <c r="F103" s="7"/>
@@ -4040,10 +4045,10 @@
       </c>
       <c r="B104" s="5"/>
       <c r="C104" s="8" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D104" s="10" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E104" s="7"/>
       <c r="F104" s="7"/>
@@ -4054,10 +4059,10 @@
       </c>
       <c r="B105" s="5"/>
       <c r="C105" s="5" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="D105" s="10" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E105" s="7"/>
       <c r="F105" s="7"/>
@@ -4068,7 +4073,7 @@
       </c>
       <c r="B106" s="5"/>
       <c r="C106" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D106" s="7"/>
       <c r="E106" s="7"/>
@@ -4079,13 +4084,13 @@
         <v>107</v>
       </c>
       <c r="B107" s="16" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C107" s="17" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D107" s="8" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="E107" s="7"/>
       <c r="F107" s="7"/>
@@ -4096,10 +4101,10 @@
       </c>
       <c r="B108" s="5"/>
       <c r="C108" s="17" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="D108" s="8" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="E108" s="7"/>
       <c r="F108" s="7"/>
@@ -4110,10 +4115,10 @@
       </c>
       <c r="B109" s="5"/>
       <c r="C109" s="17" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D109" s="8" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="E109" s="7"/>
       <c r="F109" s="7"/>
@@ -4124,10 +4129,10 @@
       </c>
       <c r="B110" s="5"/>
       <c r="C110" s="17" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D110" s="8" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E110" s="7"/>
       <c r="F110" s="7"/>
@@ -4137,13 +4142,13 @@
         <v>111</v>
       </c>
       <c r="B111" s="16" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C111" s="18" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D111" s="8" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E111" s="7"/>
       <c r="F111" s="7"/>
@@ -4154,10 +4159,10 @@
       </c>
       <c r="B112" s="5"/>
       <c r="C112" s="18" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D112" s="7" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="E112" s="7"/>
       <c r="F112" s="7"/>
@@ -4168,10 +4173,10 @@
       </c>
       <c r="B113" s="5"/>
       <c r="C113" s="18" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D113" s="7" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="E113" s="7"/>
       <c r="F113" s="7"/>
@@ -4181,13 +4186,13 @@
         <v>114</v>
       </c>
       <c r="B114" s="16" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C114" s="19" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="D114" s="8" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="E114" s="7"/>
       <c r="F114" s="7"/>
@@ -4198,10 +4203,10 @@
       </c>
       <c r="B115" s="5"/>
       <c r="C115" s="19" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D115" s="7" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="E115" s="7"/>
       <c r="F115" s="7"/>
@@ -4211,13 +4216,13 @@
         <v>116</v>
       </c>
       <c r="B116" s="16" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C116" s="20" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="D116" s="7" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E116" s="7"/>
       <c r="F116" s="7"/>
@@ -4228,10 +4233,10 @@
       </c>
       <c r="B117" s="5"/>
       <c r="C117" s="20" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="D117" s="8" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="E117" s="7"/>
       <c r="F117" s="7"/>
@@ -4242,10 +4247,10 @@
       </c>
       <c r="B118" s="5"/>
       <c r="C118" s="20" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="D118" s="8" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E118" s="7"/>
       <c r="F118" s="7"/>
@@ -4256,10 +4261,10 @@
       </c>
       <c r="B119" s="5"/>
       <c r="C119" s="20" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D119" s="7" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="E119" s="7"/>
       <c r="F119" s="7"/>
@@ -4270,10 +4275,10 @@
       </c>
       <c r="B120" s="5"/>
       <c r="C120" s="20" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D120" s="8" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E120" s="7"/>
       <c r="F120" s="7"/>
@@ -4284,10 +4289,10 @@
       </c>
       <c r="B121" s="5"/>
       <c r="C121" s="20" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D121" s="7" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E121" s="7"/>
       <c r="F121" s="7"/>
@@ -4297,13 +4302,13 @@
         <v>122</v>
       </c>
       <c r="B122" s="16" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C122" s="21" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D122" s="7" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E122" s="7"/>
       <c r="F122" s="7"/>
@@ -4314,10 +4319,10 @@
       </c>
       <c r="B123" s="5"/>
       <c r="C123" s="21" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="D123" s="7" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E123" s="7"/>
       <c r="F123" s="7"/>
@@ -4328,7 +4333,7 @@
       </c>
       <c r="B124" s="5"/>
       <c r="C124" s="6" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="D124" s="7"/>
       <c r="E124" s="7"/>
@@ -4340,13 +4345,13 @@
       </c>
       <c r="B125" s="5"/>
       <c r="C125" s="8" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D125" s="8" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="E125" s="7" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="F125" s="7"/>
     </row>
@@ -4356,13 +4361,13 @@
       </c>
       <c r="B126" s="5"/>
       <c r="C126" s="8" t="s">
+        <v>247</v>
+      </c>
+      <c r="D126" s="8" t="s">
+        <v>248</v>
+      </c>
+      <c r="E126" s="7" t="s">
         <v>246</v>
-      </c>
-      <c r="D126" s="8" t="s">
-        <v>247</v>
-      </c>
-      <c r="E126" s="7" t="s">
-        <v>245</v>
       </c>
       <c r="F126" s="7"/>
     </row>
@@ -4372,13 +4377,13 @@
       </c>
       <c r="B127" s="5"/>
       <c r="C127" s="8" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="D127" s="8" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="E127" s="7" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F127" s="7"/>
     </row>
@@ -4388,13 +4393,13 @@
       </c>
       <c r="B128" s="5"/>
       <c r="C128" s="8" t="s">
+        <v>252</v>
+      </c>
+      <c r="D128" s="8" t="s">
+        <v>253</v>
+      </c>
+      <c r="E128" s="7" t="s">
         <v>251</v>
-      </c>
-      <c r="D128" s="8" t="s">
-        <v>252</v>
-      </c>
-      <c r="E128" s="7" t="s">
-        <v>250</v>
       </c>
       <c r="F128" s="7"/>
     </row>
@@ -4404,13 +4409,13 @@
       </c>
       <c r="B129" s="5"/>
       <c r="C129" s="8" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D129" s="8" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="E129" s="7" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F129" s="7"/>
     </row>
@@ -4420,10 +4425,10 @@
       </c>
       <c r="B130" s="5"/>
       <c r="C130" s="8" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D130" s="8" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="E130" s="7"/>
       <c r="F130" s="7"/>
@@ -4434,13 +4439,13 @@
       </c>
       <c r="B131" s="5"/>
       <c r="C131" s="8" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D131" s="8" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="E131" s="7" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="F131" s="7"/>
     </row>
@@ -4450,10 +4455,10 @@
       </c>
       <c r="B132" s="5"/>
       <c r="C132" s="8" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D132" s="7" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E132" s="7"/>
       <c r="F132" s="7"/>
@@ -4464,10 +4469,10 @@
       </c>
       <c r="B133" s="5"/>
       <c r="C133" s="8" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D133" s="8" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="E133" s="7"/>
       <c r="F133" s="7"/>
@@ -4478,10 +4483,10 @@
       </c>
       <c r="B134" s="5"/>
       <c r="C134" s="5" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D134" s="7" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E134" s="7"/>
       <c r="F134" s="7"/>
@@ -4492,7 +4497,7 @@
       </c>
       <c r="B135" s="22"/>
       <c r="C135" s="6" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D135" s="22"/>
       <c r="E135" s="22"/>
@@ -4503,13 +4508,13 @@
         <v>136</v>
       </c>
       <c r="B136" s="12" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C136" s="14" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D136" s="23" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E136" s="22"/>
       <c r="F136" s="22"/>
@@ -4520,10 +4525,10 @@
       </c>
       <c r="B137" s="22"/>
       <c r="C137" s="14" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D137" s="23" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="E137" s="22"/>
       <c r="F137" s="22"/>
@@ -4534,13 +4539,13 @@
       </c>
       <c r="B138" s="22"/>
       <c r="C138" s="14" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D138" s="23" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="E138" s="14" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F138" s="22"/>
     </row>
@@ -4550,10 +4555,10 @@
       </c>
       <c r="B139" s="22"/>
       <c r="C139" s="14" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="D139" s="23" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="E139" s="22"/>
       <c r="F139" s="22"/>
@@ -4564,10 +4569,10 @@
       </c>
       <c r="B140" s="22"/>
       <c r="C140" s="14" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D140" s="23" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E140" s="22"/>
       <c r="F140" s="22"/>
@@ -4578,13 +4583,13 @@
       </c>
       <c r="B141" s="22"/>
       <c r="C141" s="14" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D141" s="23" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="E141" s="14" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F141" s="22"/>
     </row>
@@ -4593,13 +4598,13 @@
         <v>142</v>
       </c>
       <c r="B142" s="24" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C142" s="14" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D142" s="23" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="E142" s="22"/>
       <c r="F142" s="22"/>
@@ -4610,10 +4615,10 @@
       </c>
       <c r="B143" s="22"/>
       <c r="C143" s="14" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D143" s="23" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="E143" s="22"/>
       <c r="F143" s="22"/>
@@ -4624,13 +4629,13 @@
       </c>
       <c r="B144" s="22"/>
       <c r="C144" s="14" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D144" s="23" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="E144" s="14" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F144" s="22"/>
     </row>
@@ -4640,10 +4645,10 @@
       </c>
       <c r="B145" s="22"/>
       <c r="C145" s="14" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D145" s="25" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="E145" s="22"/>
       <c r="F145" s="22"/>
@@ -4654,10 +4659,10 @@
       </c>
       <c r="B146" s="22"/>
       <c r="C146" s="14" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D146" s="25" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E146" s="22"/>
       <c r="F146" s="22"/>
@@ -4667,13 +4672,13 @@
         <v>147</v>
       </c>
       <c r="B147" s="24" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C147" s="14" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D147" s="23" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="E147" s="22"/>
       <c r="F147" s="22"/>
@@ -4684,10 +4689,10 @@
       </c>
       <c r="B148" s="22"/>
       <c r="C148" s="14" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D148" s="23" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E148" s="22"/>
       <c r="F148" s="22"/>
@@ -4698,10 +4703,10 @@
       </c>
       <c r="B149" s="22"/>
       <c r="C149" s="14" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="D149" s="23" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E149" s="22"/>
       <c r="F149" s="22"/>
@@ -4712,10 +4717,10 @@
       </c>
       <c r="B150" s="22"/>
       <c r="C150" s="14" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D150" s="25" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E150" s="22"/>
       <c r="F150" s="22"/>
@@ -4726,10 +4731,10 @@
       </c>
       <c r="B151" s="22"/>
       <c r="C151" s="14" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D151" s="23" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="E151" s="22"/>
       <c r="F151" s="22"/>
@@ -4740,10 +4745,10 @@
       </c>
       <c r="B152" s="22"/>
       <c r="C152" s="14" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="D152" s="25" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="E152" s="22"/>
       <c r="F152" s="22"/>
@@ -4753,13 +4758,13 @@
         <v>153</v>
       </c>
       <c r="B153" s="24" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C153" s="14" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="D153" s="23" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="E153" s="22"/>
       <c r="F153" s="22"/>
@@ -4770,10 +4775,10 @@
       </c>
       <c r="B154" s="22"/>
       <c r="C154" s="14" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="D154" s="23" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E154" s="22"/>
       <c r="F154" s="22"/>
@@ -4784,10 +4789,10 @@
       </c>
       <c r="B155" s="22"/>
       <c r="C155" s="14" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="D155" s="23" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E155" s="22"/>
       <c r="F155" s="22"/>
@@ -4798,10 +4803,10 @@
       </c>
       <c r="B156" s="22"/>
       <c r="C156" s="14" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="D156" s="23" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E156" s="22"/>
       <c r="F156" s="22"/>
@@ -4812,10 +4817,10 @@
       </c>
       <c r="B157" s="22"/>
       <c r="C157" s="14" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="D157" s="23" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E157" s="22"/>
       <c r="F157" s="22"/>
@@ -4826,10 +4831,10 @@
       </c>
       <c r="B158" s="22"/>
       <c r="C158" s="14" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="D158" s="23" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="E158" s="22"/>
       <c r="F158" s="22"/>
@@ -4840,10 +4845,10 @@
       </c>
       <c r="B159" s="22"/>
       <c r="C159" s="14" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="D159" s="23" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="E159" s="22"/>
       <c r="F159" s="22"/>
@@ -4853,13 +4858,13 @@
         <v>160</v>
       </c>
       <c r="B160" s="24" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C160" s="14" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="D160" s="23" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="E160" s="22"/>
       <c r="F160" s="22"/>
@@ -4870,10 +4875,10 @@
       </c>
       <c r="B161" s="22"/>
       <c r="C161" s="14" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="D161" s="23" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="E161" s="22"/>
       <c r="F161" s="22"/>
@@ -4884,10 +4889,10 @@
       </c>
       <c r="B162" s="22"/>
       <c r="C162" s="14" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D162" s="23" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E162" s="22"/>
       <c r="F162" s="22"/>
@@ -4898,10 +4903,10 @@
       </c>
       <c r="B163" s="22"/>
       <c r="C163" s="14" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D163" s="25" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="E163" s="22"/>
       <c r="F163" s="22"/>
@@ -4911,13 +4916,13 @@
         <v>164</v>
       </c>
       <c r="B164" s="24" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C164" s="14" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D164" s="23" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="E164" s="22"/>
       <c r="F164" s="22"/>
@@ -4928,10 +4933,10 @@
       </c>
       <c r="B165" s="22"/>
       <c r="C165" s="14" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="D165" s="25" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="E165" s="22"/>
       <c r="F165" s="22"/>
@@ -4942,10 +4947,10 @@
       </c>
       <c r="B166" s="22"/>
       <c r="C166" s="14" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="D166" s="25" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="E166" s="22"/>
       <c r="F166" s="22"/>
@@ -4956,7 +4961,7 @@
       </c>
       <c r="B167" s="22"/>
       <c r="C167" s="26" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="D167" s="22"/>
       <c r="E167" s="22"/>
@@ -4968,10 +4973,10 @@
       </c>
       <c r="B168" s="22"/>
       <c r="C168" s="12" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="D168" s="23" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="E168" s="22"/>
       <c r="F168" s="22"/>
@@ -4982,10 +4987,10 @@
       </c>
       <c r="B169" s="22"/>
       <c r="C169" s="12" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="D169" s="23" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="E169" s="22"/>
       <c r="F169" s="22"/>
@@ -4996,10 +5001,10 @@
       </c>
       <c r="B170" s="22"/>
       <c r="C170" s="12" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D170" s="23" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="E170" s="22"/>
       <c r="F170" s="22"/>
@@ -5010,10 +5015,10 @@
       </c>
       <c r="B171" s="22"/>
       <c r="C171" s="12" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="D171" s="23" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E171" s="22"/>
       <c r="F171" s="22"/>
@@ -5024,10 +5029,10 @@
       </c>
       <c r="B172" s="22"/>
       <c r="C172" s="12" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="D172" s="23" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="E172" s="22"/>
       <c r="F172" s="22"/>
@@ -5038,10 +5043,10 @@
       </c>
       <c r="B173" s="22"/>
       <c r="C173" s="12" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="D173" s="23" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="E173" s="22"/>
       <c r="F173" s="22"/>
@@ -5052,10 +5057,10 @@
       </c>
       <c r="B174" s="22"/>
       <c r="C174" s="12" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="D174" s="23" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="E174" s="22"/>
       <c r="F174" s="22"/>
@@ -5066,10 +5071,10 @@
       </c>
       <c r="B175" s="22"/>
       <c r="C175" s="12" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="D175" s="23" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E175" s="22"/>
       <c r="F175" s="22"/>
@@ -5080,10 +5085,10 @@
       </c>
       <c r="B176" s="22"/>
       <c r="C176" s="12" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="D176" s="23" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="E176" s="22"/>
       <c r="F176" s="22"/>
@@ -5094,10 +5099,10 @@
       </c>
       <c r="B177" s="22"/>
       <c r="C177" s="12" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="D177" s="23" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="E177" s="22"/>
       <c r="F177" s="22"/>
@@ -5108,10 +5113,10 @@
       </c>
       <c r="B178" s="22"/>
       <c r="C178" s="12" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="D178" s="23" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="E178" s="22"/>
       <c r="F178" s="22"/>
@@ -5122,10 +5127,10 @@
       </c>
       <c r="B179" s="22"/>
       <c r="C179" s="12" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="D179" s="23" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="E179" s="22"/>
       <c r="F179" s="22"/>

</xml_diff>

<commit_message>
Feat: Problem 3 Remove Duplicates from array
</commit_message>
<xml_diff>
--- a/DSA Pattern sheets.xlsx
+++ b/DSA Pattern sheets.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="362">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="362">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2651,7 +2651,7 @@
       <c r="E3" s="7"/>
       <c r="F3" s="7"/>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" ht="15.15" spans="1:6">
       <c r="A4" s="4">
         <v>4</v>
       </c>
@@ -2671,7 +2671,9 @@
       <c r="A5" s="4">
         <v>5</v>
       </c>
-      <c r="B5" s="5"/>
+      <c r="B5" s="5" t="s">
+        <v>7</v>
+      </c>
       <c r="C5" s="8" t="s">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
Feat: Problem 4 sortedSquares
</commit_message>
<xml_diff>
--- a/DSA Pattern sheets.xlsx
+++ b/DSA Pattern sheets.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="362">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="362">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2667,7 +2667,7 @@
       <c r="E4" s="7"/>
       <c r="F4" s="7"/>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" ht="15.15" spans="1:6">
       <c r="A5" s="4">
         <v>5</v>
       </c>
@@ -2701,11 +2701,13 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" ht="15.15" spans="1:6">
+    <row r="7" spans="1:6">
       <c r="A7" s="4">
         <v>7</v>
       </c>
-      <c r="B7" s="5"/>
+      <c r="B7" s="5" t="s">
+        <v>7</v>
+      </c>
       <c r="C7" s="8" t="s">
         <v>16</v>
       </c>

</xml_diff>

<commit_message>
Feat: Problem 6 Remove element
</commit_message>
<xml_diff>
--- a/DSA Pattern sheets.xlsx
+++ b/DSA Pattern sheets.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="362">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="362">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2683,11 +2683,13 @@
       <c r="E5" s="8"/>
       <c r="F5" s="5"/>
     </row>
-    <row r="6" ht="15.15" spans="1:6">
+    <row r="6" spans="1:6">
       <c r="A6" s="4">
         <v>6</v>
       </c>
-      <c r="B6" s="5"/>
+      <c r="B6" s="5" t="s">
+        <v>7</v>
+      </c>
       <c r="C6" s="8" t="s">
         <v>12</v>
       </c>
@@ -2701,7 +2703,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" ht="15.15" spans="1:6">
       <c r="A7" s="4">
         <v>7</v>
       </c>

</xml_diff>

<commit_message>
Feat: Problem 8 Sort Colors
</commit_message>
<xml_diff>
--- a/DSA Pattern sheets.xlsx
+++ b/DSA Pattern sheets.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="362">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="373" uniqueCount="362">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2683,7 +2683,7 @@
       <c r="E5" s="8"/>
       <c r="F5" s="5"/>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" ht="15.15" spans="1:6">
       <c r="A6" s="4">
         <v>6</v>
       </c>
@@ -2719,11 +2719,13 @@
       <c r="E7" s="7"/>
       <c r="F7" s="7"/>
     </row>
-    <row r="8" ht="15.15" spans="1:6">
+    <row r="8" spans="1:6">
       <c r="A8" s="4">
         <v>8</v>
       </c>
-      <c r="B8" s="5"/>
+      <c r="B8" s="5" t="s">
+        <v>7</v>
+      </c>
       <c r="C8" s="8" t="s">
         <v>18</v>
       </c>

</xml_diff>